<commit_message>
Perbarui data SE2026 29/08/2026 16:23:49,84
</commit_message>
<xml_diff>
--- a/data/20260823_125317_Radar_Anomali_Keluarga_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Kabupaten_Kota.xlsx
+++ b/data/20260823_125317_Radar_Anomali_Keluarga_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="306">
   <si>
     <t>DATA RADAR ANOMALI KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 28 Agu 2026, 10.22</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 29 Agu 2026, 16.20</t>
   </si>
   <si>
     <t>Kode</t>
@@ -298,604 +298,631 @@
     <t>0,01</t>
   </si>
   <si>
-    <t>4,17</t>
+    <t>4,19</t>
+  </si>
+  <si>
+    <t>0,68</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>19,66</t>
+  </si>
+  <si>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>0,69</t>
+  </si>
+  <si>
+    <t>2,44</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>2,87</t>
+  </si>
+  <si>
+    <t>0,55</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>43,28</t>
+  </si>
+  <si>
+    <t>1,04</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>16,58</t>
+  </si>
+  <si>
+    <t>6,99</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>3,82</t>
+  </si>
+  <si>
+    <t>0,97</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>25,85</t>
   </si>
   <si>
     <t>0,7</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>19,37</t>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>1,52</t>
+  </si>
+  <si>
+    <t>4,09</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>38,27</t>
+  </si>
+  <si>
+    <t>0,52</t>
+  </si>
+  <si>
+    <t>12,27</t>
+  </si>
+  <si>
+    <t>11,52</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>19,78</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>0,9</t>
+  </si>
+  <si>
+    <t>3,31</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>3,19</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>41,85</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>22,73</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>5,81</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>19,03</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>3,25</t>
+  </si>
+  <si>
+    <t>3,35</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>43,81</t>
+  </si>
+  <si>
+    <t>3,96</t>
+  </si>
+  <si>
+    <t>17,86</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>4,36</t>
+  </si>
+  <si>
+    <t>24,87</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>2,7</t>
+  </si>
+  <si>
+    <t>0,29</t>
+  </si>
+  <si>
+    <t>3,38</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>1,76</t>
+  </si>
+  <si>
+    <t>42,99</t>
+  </si>
+  <si>
+    <t>0,41</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>15,19</t>
+  </si>
+  <si>
+    <t>1,73</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>4,2</t>
+  </si>
+  <si>
+    <t>22,04</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>5,84</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>44,87</t>
+  </si>
+  <si>
+    <t>1,18</t>
+  </si>
+  <si>
+    <t>15,18</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>2,58</t>
+  </si>
+  <si>
+    <t>2,3</t>
+  </si>
+  <si>
+    <t>14,39</t>
+  </si>
+  <si>
+    <t>0,05</t>
   </si>
   <si>
     <t>0,44</t>
   </si>
   <si>
-    <t>2,46</t>
-  </si>
-  <si>
-    <t>0,27</t>
-  </si>
-  <si>
-    <t>2,89</t>
-  </si>
-  <si>
-    <t>0,55</t>
-  </si>
-  <si>
-    <t>0,35</t>
-  </si>
-  <si>
-    <t>43,08</t>
-  </si>
-  <si>
-    <t>1,06</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>16,67</t>
-  </si>
-  <si>
-    <t>7,19</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>3,59</t>
-  </si>
-  <si>
-    <t>1,03</t>
-  </si>
-  <si>
-    <t>24,82</t>
-  </si>
-  <si>
-    <t>0,74</t>
+    <t>2,25</t>
+  </si>
+  <si>
+    <t>44,38</t>
+  </si>
+  <si>
+    <t>0,79</t>
+  </si>
+  <si>
+    <t>16,75</t>
+  </si>
+  <si>
+    <t>12,92</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>4,33</t>
+  </si>
+  <si>
+    <t>20,04</t>
   </si>
   <si>
     <t>0,13</t>
   </si>
   <si>
-    <t>1,6</t>
-  </si>
-  <si>
-    <t>4,23</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>38,42</t>
-  </si>
-  <si>
-    <t>12,32</t>
-  </si>
-  <si>
-    <t>12,19</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>6,57</t>
-  </si>
-  <si>
-    <t>19,6</t>
-  </si>
-  <si>
-    <t>0,3</t>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>2,48</t>
+  </si>
+  <si>
+    <t>2,95</t>
+  </si>
+  <si>
+    <t>0,38</t>
+  </si>
+  <si>
+    <t>41,25</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>26,1</t>
+  </si>
+  <si>
+    <t>1,22</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>0,78</t>
+  </si>
+  <si>
+    <t>21,49</t>
+  </si>
+  <si>
+    <t>0,92</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>2,16</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>2,02</t>
+  </si>
+  <si>
+    <t>46,37</t>
+  </si>
+  <si>
+    <t>15,43</t>
+  </si>
+  <si>
+    <t>4,55</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>3,29</t>
+  </si>
+  <si>
+    <t>13,41</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>1,26</t>
+  </si>
+  <si>
+    <t>40,61</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>14,7</t>
+  </si>
+  <si>
+    <t>22,05</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>4,98</t>
+  </si>
+  <si>
+    <t>15,15</t>
+  </si>
+  <si>
+    <t>0,65</t>
+  </si>
+  <si>
+    <t>1,41</t>
+  </si>
+  <si>
+    <t>5,08</t>
+  </si>
+  <si>
+    <t>4,13</t>
+  </si>
+  <si>
+    <t>1,01</t>
   </si>
   <si>
     <t>0,91</t>
   </si>
   <si>
-    <t>3,35</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>3,23</t>
-  </si>
-  <si>
-    <t>41,75</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>22,7</t>
+    <t>43,18</t>
+  </si>
+  <si>
+    <t>1,61</t>
+  </si>
+  <si>
+    <t>18,52</t>
+  </si>
+  <si>
+    <t>2,82</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>0,82</t>
+  </si>
+  <si>
+    <t>20,42</t>
+  </si>
+  <si>
+    <t>0,73</t>
+  </si>
+  <si>
+    <t>0,89</t>
+  </si>
+  <si>
+    <t>1,55</t>
+  </si>
+  <si>
+    <t>49,04</t>
+  </si>
+  <si>
+    <t>1,33</t>
+  </si>
+  <si>
+    <t>12,46</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>4,15</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>20,71</t>
+  </si>
+  <si>
+    <t>0,51</t>
+  </si>
+  <si>
+    <t>0,48</t>
+  </si>
+  <si>
+    <t>1,62</t>
+  </si>
+  <si>
+    <t>0,17</t>
+  </si>
+  <si>
+    <t>1,64</t>
+  </si>
+  <si>
+    <t>45,67</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>23,03</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>4,45</t>
+  </si>
+  <si>
+    <t>26,53</t>
   </si>
   <si>
     <t>0,43</t>
   </si>
   <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>5,83</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>18,98</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>3,28</t>
-  </si>
-  <si>
-    <t>3,37</t>
-  </si>
-  <si>
-    <t>0,75</t>
-  </si>
-  <si>
-    <t>43,73</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>17,82</t>
-  </si>
-  <si>
-    <t>1,16</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>4,28</t>
-  </si>
-  <si>
-    <t>0,4</t>
-  </si>
-  <si>
-    <t>24,63</t>
-  </si>
-  <si>
-    <t>0,31</t>
-  </si>
-  <si>
-    <t>1,23</t>
-  </si>
-  <si>
-    <t>2,99</t>
+    <t>3,34</t>
+  </si>
+  <si>
+    <t>43,25</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>16,62</t>
+  </si>
+  <si>
+    <t>3,69</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>6,96</t>
+  </si>
+  <si>
+    <t>9,18</t>
+  </si>
+  <si>
+    <t>6,49</t>
+  </si>
+  <si>
+    <t>2,53</t>
+  </si>
+  <si>
+    <t>7,28</t>
+  </si>
+  <si>
+    <t>13,92</t>
+  </si>
+  <si>
+    <t>36,55</t>
+  </si>
+  <si>
+    <t>1,9</t>
+  </si>
+  <si>
+    <t>9,02</t>
+  </si>
+  <si>
+    <t>3,01</t>
   </si>
   <si>
     <t>0,32</t>
   </si>
   <si>
-    <t>3,6</t>
-  </si>
-  <si>
-    <t>1,97</t>
-  </si>
-  <si>
-    <t>42,12</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>15,18</t>
-  </si>
-  <si>
-    <t>1,92</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>4,25</t>
-  </si>
-  <si>
-    <t>22,01</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>5,9</t>
-  </si>
-  <si>
-    <t>4,18</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>44,74</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>15,2</t>
-  </si>
-  <si>
-    <t>0,64</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>2,58</t>
-  </si>
-  <si>
-    <t>2,31</t>
-  </si>
-  <si>
-    <t>14,4</t>
-  </si>
-  <si>
-    <t>2,25</t>
-  </si>
-  <si>
-    <t>2,44</t>
-  </si>
-  <si>
-    <t>44,38</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>16,73</t>
-  </si>
-  <si>
-    <t>12,93</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>20,1</t>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>2,45</t>
+  </si>
+  <si>
+    <t>11,56</t>
   </si>
   <si>
     <t>0,61</t>
   </si>
   <si>
-    <t>2,53</t>
-  </si>
-  <si>
-    <t>2,95</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>40,93</t>
-  </si>
-  <si>
-    <t>26,35</t>
-  </si>
-  <si>
-    <t>1,25</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>4,32</t>
-  </si>
-  <si>
-    <t>0,78</t>
-  </si>
-  <si>
-    <t>21,44</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>1,2</t>
-  </si>
-  <si>
-    <t>2,16</t>
-  </si>
-  <si>
-    <t>2,02</t>
-  </si>
-  <si>
-    <t>46,41</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>15,46</t>
-  </si>
-  <si>
-    <t>4,55</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>3,27</t>
-  </si>
-  <si>
-    <t>1,15</t>
-  </si>
-  <si>
-    <t>13,33</t>
-  </si>
-  <si>
-    <t>0,58</t>
-  </si>
-  <si>
-    <t>0,94</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>1,24</t>
-  </si>
-  <si>
-    <t>40,55</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>14,73</t>
-  </si>
-  <si>
-    <t>22,17</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>5,01</t>
-  </si>
-  <si>
-    <t>14,61</t>
-  </si>
-  <si>
-    <t>1,81</t>
-  </si>
-  <si>
-    <t>4,34</t>
-  </si>
-  <si>
-    <t>0,57</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>43,21</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>18,33</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>4,44</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>19,85</t>
-  </si>
-  <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>1,53</t>
-  </si>
-  <si>
-    <t>48,91</t>
-  </si>
-  <si>
-    <t>1,34</t>
-  </si>
-  <si>
-    <t>12,7</t>
-  </si>
-  <si>
-    <t>7,22</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>4,16</t>
-  </si>
-  <si>
-    <t>20,18</t>
-  </si>
-  <si>
-    <t>0,88</t>
-  </si>
-  <si>
-    <t>0,5</t>
-  </si>
-  <si>
-    <t>1,51</t>
-  </si>
-  <si>
-    <t>45,49</t>
+    <t>2,38</t>
+  </si>
+  <si>
+    <t>2,52</t>
+  </si>
+  <si>
+    <t>2,65</t>
+  </si>
+  <si>
+    <t>1,09</t>
+  </si>
+  <si>
+    <t>41,84</t>
   </si>
   <si>
     <t>0,2</t>
   </si>
   <si>
-    <t>23,55</t>
-  </si>
-  <si>
-    <t>1,01</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>4,46</t>
-  </si>
-  <si>
-    <t>26,59</t>
-  </si>
-  <si>
-    <t>3,44</t>
-  </si>
-  <si>
-    <t>42,56</t>
-  </si>
-  <si>
-    <t>0,68</t>
-  </si>
-  <si>
-    <t>16,94</t>
-  </si>
-  <si>
-    <t>3,83</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>6,97</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>9,19</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>6,5</t>
-  </si>
-  <si>
-    <t>2,54</t>
-  </si>
-  <si>
-    <t>7,13</t>
-  </si>
-  <si>
-    <t>13,95</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>36,61</t>
-  </si>
-  <si>
-    <t>1,9</t>
-  </si>
-  <si>
-    <t>9,03</t>
-  </si>
-  <si>
-    <t>3,01</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>2,32</t>
-  </si>
-  <si>
-    <t>0,41</t>
-  </si>
-  <si>
-    <t>11,48</t>
-  </si>
-  <si>
-    <t>2,39</t>
-  </si>
-  <si>
-    <t>2,66</t>
-  </si>
-  <si>
-    <t>41,8</t>
-  </si>
-  <si>
-    <t>8,13</t>
-  </si>
-  <si>
-    <t>26,23</t>
+    <t>8,1</t>
+  </si>
+  <si>
+    <t>26,12</t>
   </si>
   <si>
     <t/>
@@ -1821,7 +1848,7 @@
         <v>93</v>
       </c>
       <c r="C6" s="6">
-        <v>56632</v>
+        <v>58216</v>
       </c>
       <c r="D6" s="6">
         <v>7</v>
@@ -1830,7 +1857,7 @@
         <v>94</v>
       </c>
       <c r="F6" s="6">
-        <v>2361</v>
+        <v>2441</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>95</v>
@@ -1848,7 +1875,7 @@
         <v>97</v>
       </c>
       <c r="L6" s="6">
-        <v>10972</v>
+        <v>11446</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>98</v>
@@ -1860,76 +1887,76 @@
         <v>94</v>
       </c>
       <c r="P6" s="6">
-        <v>251</v>
+        <v>211</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>99</v>
       </c>
       <c r="R6" s="6">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="T6" s="6">
-        <v>1391</v>
+        <v>1423</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="V6" s="6">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="W6" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="X6" s="6">
-        <v>1637</v>
+        <v>1670</v>
       </c>
       <c r="Y6" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="Z6" s="6">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="AA6" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AB6" s="6">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="AC6" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AD6" s="6">
-        <v>24396</v>
+        <v>25193</v>
       </c>
       <c r="AE6" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AF6" s="6">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="AG6" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AH6" s="6">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AI6" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AJ6" s="6">
-        <v>9441</v>
+        <v>9655</v>
       </c>
       <c r="AK6" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AL6" s="6">
         <v>4070</v>
       </c>
       <c r="AM6" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AN6" s="6">
         <v>4</v>
@@ -1947,18 +1974,18 @@
         <v>26</v>
       </c>
       <c r="AS6" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C7" s="9">
-        <v>3118</v>
+        <v>3300</v>
       </c>
       <c r="D7" s="9">
         <v>0</v>
@@ -1967,28 +1994,28 @@
         <v>97</v>
       </c>
       <c r="F7" s="9">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H7" s="9">
         <v>32</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J7" s="9">
         <v>1</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="L7" s="9">
-        <v>774</v>
+        <v>853</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="N7" s="9">
         <v>0</v>
@@ -2000,73 +2027,73 @@
         <v>23</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="R7" s="9">
         <v>4</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="T7" s="9">
         <v>4</v>
       </c>
       <c r="U7" s="10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="V7" s="9">
         <v>50</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="X7" s="9">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="Z7" s="9">
         <v>3</v>
       </c>
       <c r="AA7" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="AB7" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC7" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AD7" s="9">
-        <v>1198</v>
+        <v>1263</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="AF7" s="9">
         <v>17</v>
       </c>
       <c r="AG7" s="10" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="AH7" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI7" s="10" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="AJ7" s="9">
-        <v>384</v>
+        <v>405</v>
       </c>
       <c r="AK7" s="10" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AL7" s="9">
         <v>380</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AN7" s="9">
         <v>0</v>
@@ -2089,13 +2116,13 @@
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C8" s="9">
-        <v>1643</v>
+        <v>1663</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2104,10 +2131,10 @@
         <v>97</v>
       </c>
       <c r="F8" s="9">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H8" s="9">
         <v>0</v>
@@ -2122,10 +2149,10 @@
         <v>97</v>
       </c>
       <c r="L8" s="9">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="N8" s="9">
         <v>0</v>
@@ -2134,76 +2161,76 @@
         <v>97</v>
       </c>
       <c r="P8" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="R8" s="9">
         <v>15</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="T8" s="9">
         <v>55</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="V8" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="X8" s="9">
         <v>53</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="Z8" s="9">
         <v>5</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="AB8" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="AD8" s="9">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AF8" s="9">
         <v>2</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="AH8" s="9">
         <v>1</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AJ8" s="9">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AL8" s="9">
         <v>7</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
@@ -2221,36 +2248,36 @@
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C9" s="9">
-        <v>5881</v>
+        <v>5939</v>
       </c>
       <c r="D9" s="9">
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
       <c r="F9" s="9">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H9" s="9">
         <v>22</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J9" s="9">
         <v>0</v>
@@ -2259,10 +2286,10 @@
         <v>97</v>
       </c>
       <c r="L9" s="9">
-        <v>1116</v>
+        <v>1130</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="N9" s="9">
         <v>0</v>
@@ -2271,40 +2298,40 @@
         <v>97</v>
       </c>
       <c r="P9" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="R9" s="9">
         <v>33</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="T9" s="9">
         <v>193</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="V9" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="X9" s="9">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="Z9" s="9">
         <v>44</v>
       </c>
       <c r="AA9" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="AB9" s="9">
         <v>0</v>
@@ -2313,16 +2340,16 @@
         <v>97</v>
       </c>
       <c r="AD9" s="9">
-        <v>2572</v>
+        <v>2602</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="AF9" s="9">
         <v>235</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
@@ -2331,16 +2358,16 @@
         <v>97</v>
       </c>
       <c r="AJ9" s="9">
-        <v>1048</v>
+        <v>1061</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AL9" s="9">
         <v>68</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
@@ -2358,36 +2385,36 @@
         <v>4</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C10" s="9">
-        <v>6192</v>
+        <v>6859</v>
       </c>
       <c r="D10" s="9">
         <v>3</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F10" s="9">
-        <v>265</v>
+        <v>299</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H10" s="9">
         <v>25</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>156</v>
+        <v>99</v>
       </c>
       <c r="J10" s="9">
         <v>0</v>
@@ -2396,94 +2423,94 @@
         <v>97</v>
       </c>
       <c r="L10" s="9">
-        <v>1525</v>
+        <v>1706</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N10" s="9">
         <v>1</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>140</v>
+        <v>94</v>
       </c>
       <c r="P10" s="9">
         <v>19</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="R10" s="9">
         <v>76</v>
       </c>
       <c r="S10" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="T10" s="9">
         <v>185</v>
       </c>
       <c r="U10" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="V10" s="9">
         <v>20</v>
       </c>
       <c r="W10" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="X10" s="9">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="Z10" s="9">
         <v>23</v>
       </c>
       <c r="AA10" s="10" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="AB10" s="9">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AC10" s="10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AD10" s="9">
-        <v>2608</v>
+        <v>2949</v>
       </c>
       <c r="AE10" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="AF10" s="9">
         <v>28</v>
       </c>
       <c r="AG10" s="10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="AH10" s="9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AI10" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="AJ10" s="9">
-        <v>940</v>
+        <v>1042</v>
       </c>
       <c r="AK10" s="10" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="AL10" s="9">
         <v>119</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="AN10" s="9">
         <v>1</v>
       </c>
       <c r="AO10" s="10" t="s">
-        <v>140</v>
+        <v>94</v>
       </c>
       <c r="AP10" s="9">
         <v>0</v>
@@ -2495,36 +2522,36 @@
         <v>3</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C11" s="9">
-        <v>6120</v>
+        <v>6185</v>
       </c>
       <c r="D11" s="9">
         <v>2</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F11" s="9">
         <v>260</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H11" s="9">
         <v>6</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="J11" s="9">
         <v>0</v>
@@ -2533,10 +2560,10 @@
         <v>97</v>
       </c>
       <c r="L11" s="9">
-        <v>1347</v>
+        <v>1363</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="N11" s="9">
         <v>0</v>
@@ -2548,55 +2575,55 @@
         <v>34</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>144</v>
+        <v>104</v>
       </c>
       <c r="R11" s="9">
         <v>28</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T11" s="9">
         <v>361</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="V11" s="9">
         <v>6</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="X11" s="9">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>174</v>
+        <v>95</v>
       </c>
       <c r="Z11" s="9">
         <v>29</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AB11" s="9">
         <v>9</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AD11" s="9">
-        <v>2738</v>
+        <v>2775</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="AF11" s="9">
         <v>73</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AH11" s="9">
         <v>0</v>
@@ -2605,16 +2632,16 @@
         <v>97</v>
       </c>
       <c r="AJ11" s="9">
-        <v>930</v>
+        <v>939</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AL11" s="9">
         <v>39</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="AN11" s="9">
         <v>0</v>
@@ -2632,18 +2659,18 @@
         <v>2</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C12" s="9">
-        <v>5856</v>
+        <v>5858</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
@@ -2655,13 +2682,13 @@
         <v>151</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H12" s="9">
         <v>135</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J12" s="9">
         <v>0</v>
@@ -2673,7 +2700,7 @@
         <v>843</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="N12" s="9">
         <v>0</v>
@@ -2685,37 +2712,37 @@
         <v>3</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
       <c r="R12" s="9">
         <v>26</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>99</v>
+        <v>189</v>
       </c>
       <c r="T12" s="9">
         <v>132</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="V12" s="9">
         <v>2</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="X12" s="9">
         <v>143</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>187</v>
+        <v>101</v>
       </c>
       <c r="Z12" s="9">
         <v>32</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
@@ -2724,16 +2751,16 @@
         <v>97</v>
       </c>
       <c r="AD12" s="9">
-        <v>2599</v>
+        <v>2600</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AF12" s="9">
         <v>46</v>
       </c>
       <c r="AG12" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AH12" s="9">
         <v>0</v>
@@ -2742,22 +2769,22 @@
         <v>97</v>
       </c>
       <c r="AJ12" s="9">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="AK12" s="10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="AL12" s="9">
         <v>757</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="AN12" s="9">
         <v>1</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
       <c r="AP12" s="9">
         <v>0</v>
@@ -2769,18 +2796,18 @@
         <v>6</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C13" s="9">
-        <v>3120</v>
+        <v>3188</v>
       </c>
       <c r="D13" s="9">
         <v>0</v>
@@ -2789,16 +2816,16 @@
         <v>97</v>
       </c>
       <c r="F13" s="9">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>119</v>
+        <v>197</v>
       </c>
       <c r="H13" s="9">
         <v>2</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="J13" s="9">
         <v>0</v>
@@ -2807,70 +2834,70 @@
         <v>97</v>
       </c>
       <c r="L13" s="9">
-        <v>627</v>
+        <v>639</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="N13" s="9">
         <v>1</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="P13" s="9">
         <v>4</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>117</v>
+        <v>199</v>
       </c>
       <c r="R13" s="9">
         <v>19</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="T13" s="9">
         <v>79</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="V13" s="9">
         <v>3</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="X13" s="9">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="Z13" s="9">
         <v>12</v>
       </c>
       <c r="AA13" s="10" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="AB13" s="9">
         <v>1</v>
       </c>
       <c r="AC13" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="AD13" s="9">
-        <v>1277</v>
+        <v>1315</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="AF13" s="9">
         <v>10</v>
       </c>
       <c r="AG13" s="10" t="s">
-        <v>161</v>
+        <v>205</v>
       </c>
       <c r="AH13" s="9">
         <v>0</v>
@@ -2879,16 +2906,16 @@
         <v>97</v>
       </c>
       <c r="AJ13" s="9">
-        <v>822</v>
+        <v>832</v>
       </c>
       <c r="AK13" s="10" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="AL13" s="9">
         <v>39</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="AN13" s="9">
         <v>0</v>
@@ -2911,13 +2938,13 @@
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="C14" s="9">
-        <v>2174</v>
+        <v>2178</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
@@ -2926,16 +2953,16 @@
         <v>97</v>
       </c>
       <c r="F14" s="9">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>204</v>
+        <v>157</v>
       </c>
       <c r="H14" s="9">
         <v>17</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="J14" s="9">
         <v>0</v>
@@ -2944,52 +2971,52 @@
         <v>97</v>
       </c>
       <c r="L14" s="9">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="N14" s="9">
         <v>1</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
       <c r="P14" s="9">
         <v>20</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="R14" s="9">
         <v>26</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="T14" s="9">
         <v>47</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="V14" s="9">
         <v>10</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>172</v>
+        <v>215</v>
       </c>
       <c r="X14" s="9">
         <v>44</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
@@ -2998,16 +3025,16 @@
         <v>97</v>
       </c>
       <c r="AD14" s="9">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="AF14" s="9">
         <v>2</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>212</v>
+        <v>122</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
@@ -3019,19 +3046,19 @@
         <v>336</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="AL14" s="9">
         <v>99</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="AN14" s="9">
         <v>1</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
       <c r="AP14" s="9">
         <v>0</v>
@@ -3043,18 +3070,18 @@
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C15" s="9">
-        <v>7650</v>
+        <v>7693</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -3063,16 +3090,16 @@
         <v>97</v>
       </c>
       <c r="F15" s="9">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="H15" s="9">
         <v>88</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>218</v>
+        <v>153</v>
       </c>
       <c r="J15" s="9">
         <v>0</v>
@@ -3081,10 +3108,10 @@
         <v>97</v>
       </c>
       <c r="L15" s="9">
-        <v>1020</v>
+        <v>1032</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="N15" s="9">
         <v>0</v>
@@ -3093,40 +3120,40 @@
         <v>97</v>
       </c>
       <c r="P15" s="9">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>220</v>
+        <v>104</v>
       </c>
       <c r="R15" s="9">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="T15" s="9">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="V15" s="9">
         <v>4</v>
       </c>
       <c r="W15" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
       <c r="X15" s="9">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Y15" s="10" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="Z15" s="9">
         <v>8</v>
       </c>
       <c r="AA15" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="AB15" s="9">
         <v>0</v>
@@ -3135,16 +3162,16 @@
         <v>97</v>
       </c>
       <c r="AD15" s="9">
-        <v>3102</v>
+        <v>3124</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="AF15" s="9">
         <v>66</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="AH15" s="9">
         <v>0</v>
@@ -3153,16 +3180,16 @@
         <v>97</v>
       </c>
       <c r="AJ15" s="9">
-        <v>1127</v>
+        <v>1131</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="AL15" s="9">
         <v>1696</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="AN15" s="9">
         <v>1</v>
@@ -3180,18 +3207,18 @@
         <v>2</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C16" s="9">
-        <v>1937</v>
+        <v>1987</v>
       </c>
       <c r="D16" s="9">
         <v>0</v>
@@ -3200,16 +3227,16 @@
         <v>97</v>
       </c>
       <c r="F16" s="9">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="H16" s="9">
         <v>6</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="J16" s="9">
         <v>0</v>
@@ -3218,10 +3245,10 @@
         <v>97</v>
       </c>
       <c r="L16" s="9">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="N16" s="9">
         <v>0</v>
@@ -3230,76 +3257,76 @@
         <v>97</v>
       </c>
       <c r="P16" s="9">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="R16" s="9">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="S16" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="T16" s="9">
+        <v>101</v>
+      </c>
+      <c r="U16" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="V16" s="9">
+        <v>0</v>
+      </c>
+      <c r="W16" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="X16" s="9">
+        <v>82</v>
+      </c>
+      <c r="Y16" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="Z16" s="9">
+        <v>20</v>
+      </c>
+      <c r="AA16" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="AB16" s="9">
+        <v>18</v>
+      </c>
+      <c r="AC16" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="AD16" s="9">
+        <v>858</v>
+      </c>
+      <c r="AE16" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="AF16" s="9">
+        <v>32</v>
+      </c>
+      <c r="AG16" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="AH16" s="9">
+        <v>3</v>
+      </c>
+      <c r="AI16" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="T16" s="9">
-        <v>84</v>
-      </c>
-      <c r="U16" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="V16" s="9">
-        <v>9</v>
-      </c>
-      <c r="W16" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="X16" s="9">
-        <v>81</v>
-      </c>
-      <c r="Y16" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z16" s="9">
-        <v>11</v>
-      </c>
-      <c r="AA16" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="AB16" s="9">
-        <v>22</v>
-      </c>
-      <c r="AC16" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="AD16" s="9">
-        <v>837</v>
-      </c>
-      <c r="AE16" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="AF16" s="9">
-        <v>31</v>
-      </c>
-      <c r="AG16" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH16" s="9">
-        <v>5</v>
-      </c>
-      <c r="AI16" s="10" t="s">
-        <v>237</v>
-      </c>
       <c r="AJ16" s="9">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="AL16" s="9">
         <v>56</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>102</v>
+        <v>244</v>
       </c>
       <c r="AN16" s="9">
         <v>0</v>
@@ -3317,36 +3344,36 @@
         <v>2</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C17" s="9">
-        <v>3063</v>
+        <v>3163</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F17" s="9">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>241</v>
+        <v>157</v>
       </c>
       <c r="H17" s="9">
         <v>26</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="J17" s="9">
         <v>0</v>
@@ -3355,10 +3382,10 @@
         <v>97</v>
       </c>
       <c r="L17" s="9">
-        <v>608</v>
+        <v>646</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="N17" s="9">
         <v>0</v>
@@ -3370,73 +3397,73 @@
         <v>23</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>147</v>
+        <v>249</v>
       </c>
       <c r="R17" s="9">
         <v>28</v>
       </c>
       <c r="S17" s="10" t="s">
-        <v>129</v>
+        <v>250</v>
       </c>
       <c r="T17" s="9">
         <v>30</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="V17" s="9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>244</v>
+        <v>159</v>
       </c>
       <c r="X17" s="9">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="Z17" s="9">
         <v>2</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="AD17" s="9">
-        <v>1498</v>
+        <v>1551</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="AF17" s="9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AG17" s="10" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="AH17" s="9">
         <v>1</v>
       </c>
       <c r="AI17" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="AJ17" s="9">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="AK17" s="10" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="AL17" s="9">
         <v>221</v>
       </c>
       <c r="AM17" s="10" t="s">
-        <v>249</v>
+        <v>110</v>
       </c>
       <c r="AN17" s="9">
         <v>0</v>
@@ -3459,13 +3486,13 @@
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C18" s="9">
-        <v>3970</v>
+        <v>4143</v>
       </c>
       <c r="D18" s="9">
         <v>0</v>
@@ -3474,16 +3501,16 @@
         <v>97</v>
       </c>
       <c r="F18" s="9">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="H18" s="9">
         <v>6</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>176</v>
+        <v>258</v>
       </c>
       <c r="J18" s="9">
         <v>0</v>
@@ -3492,10 +3519,10 @@
         <v>97</v>
       </c>
       <c r="L18" s="9">
-        <v>801</v>
+        <v>858</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="N18" s="9">
         <v>0</v>
@@ -3504,76 +3531,76 @@
         <v>97</v>
       </c>
       <c r="P18" s="9">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="R18" s="9">
         <v>20</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="T18" s="9">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="V18" s="9">
+        <v>7</v>
+      </c>
+      <c r="W18" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="X18" s="9">
+        <v>68</v>
+      </c>
+      <c r="Y18" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="Z18" s="9">
         <v>13</v>
       </c>
-      <c r="W18" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="X18" s="9">
-        <v>60</v>
-      </c>
-      <c r="Y18" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="Z18" s="9">
-        <v>12</v>
-      </c>
       <c r="AA18" s="10" t="s">
-        <v>128</v>
+        <v>205</v>
       </c>
       <c r="AB18" s="9">
         <v>15</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="AD18" s="9">
-        <v>1806</v>
+        <v>1892</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="AF18" s="9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="AH18" s="9">
         <v>1</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AJ18" s="9">
-        <v>935</v>
+        <v>954</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="AL18" s="9">
         <v>40</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>260</v>
+        <v>115</v>
       </c>
       <c r="AN18" s="9">
         <v>0</v>
@@ -3596,13 +3623,13 @@
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="C19" s="9">
-        <v>3813</v>
+        <v>3958</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
@@ -3611,10 +3638,10 @@
         <v>97</v>
       </c>
       <c r="F19" s="9">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="H19" s="9">
         <v>18</v>
@@ -3629,10 +3656,10 @@
         <v>97</v>
       </c>
       <c r="L19" s="9">
-        <v>1014</v>
+        <v>1050</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="N19" s="9">
         <v>0</v>
@@ -3647,16 +3674,16 @@
         <v>97</v>
       </c>
       <c r="R19" s="9">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>142</v>
+        <v>203</v>
       </c>
       <c r="T19" s="9">
         <v>17</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>165</v>
+        <v>272</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
@@ -3665,52 +3692,52 @@
         <v>97</v>
       </c>
       <c r="X19" s="9">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="Z19" s="9">
         <v>4</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="AB19" s="9">
         <v>1</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="AD19" s="9">
-        <v>1623</v>
+        <v>1712</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="AF19" s="9">
         <v>26</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="AH19" s="9">
         <v>1</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="AJ19" s="9">
-        <v>646</v>
+        <v>658</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="AL19" s="9">
         <v>146</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
@@ -3728,18 +3755,18 @@
         <v>2</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>110</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="C20" s="9">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
@@ -3751,13 +3778,13 @@
         <v>44</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>273</v>
+        <v>224</v>
       </c>
       <c r="J20" s="9">
         <v>0</v>
@@ -3769,7 +3796,7 @@
         <v>58</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="N20" s="9">
         <v>0</v>
@@ -3781,55 +3808,55 @@
         <v>5</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="R20" s="9">
         <v>4</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>275</v>
+        <v>182</v>
       </c>
       <c r="T20" s="9">
         <v>41</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="V20" s="9">
         <v>16</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="X20" s="9">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="Z20" s="9">
         <v>88</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="AB20" s="9">
         <v>3</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>280</v>
+        <v>177</v>
       </c>
       <c r="AD20" s="9">
         <v>231</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="AF20" s="9">
         <v>12</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="AH20" s="9">
         <v>0</v>
@@ -3841,13 +3868,13 @@
         <v>57</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="AL20" s="9">
         <v>19</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="AN20" s="9">
         <v>0</v>
@@ -3865,18 +3892,18 @@
         <v>2</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>161</v>
+        <v>290</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="C21" s="9">
-        <v>1464</v>
+        <v>1470</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
@@ -3885,16 +3912,16 @@
         <v>97</v>
       </c>
       <c r="F21" s="9">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H21" s="9">
         <v>6</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>288</v>
+        <v>167</v>
       </c>
       <c r="J21" s="9">
         <v>0</v>
@@ -3903,10 +3930,10 @@
         <v>97</v>
       </c>
       <c r="L21" s="9">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="N21" s="9">
         <v>0</v>
@@ -3924,49 +3951,49 @@
         <v>9</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>195</v>
+        <v>295</v>
       </c>
       <c r="T21" s="9">
         <v>35</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="V21" s="9">
         <v>1</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="X21" s="9">
         <v>37</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>196</v>
+        <v>297</v>
       </c>
       <c r="Z21" s="9">
         <v>39</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="AB21" s="9">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>151</v>
+        <v>299</v>
       </c>
       <c r="AD21" s="9">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="AF21" s="9">
         <v>3</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>258</v>
+        <v>301</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
@@ -3978,13 +4005,13 @@
         <v>119</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="AL21" s="9">
         <v>384</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
@@ -4007,13 +4034,13 @@
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="C22" s="12">
-        <v>56632</v>
+        <v>58216</v>
       </c>
       <c r="D22" s="12">
         <v>7</v>
@@ -4022,7 +4049,7 @@
         <v>94</v>
       </c>
       <c r="F22" s="12">
-        <v>2361</v>
+        <v>2441</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>95</v>
@@ -4040,7 +4067,7 @@
         <v>97</v>
       </c>
       <c r="L22" s="12">
-        <v>10972</v>
+        <v>11446</v>
       </c>
       <c r="M22" s="13" t="s">
         <v>98</v>
@@ -4052,76 +4079,76 @@
         <v>94</v>
       </c>
       <c r="P22" s="12">
-        <v>251</v>
+        <v>211</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>99</v>
       </c>
       <c r="R22" s="12">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="S22" s="13" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="T22" s="12">
-        <v>1391</v>
+        <v>1423</v>
       </c>
       <c r="U22" s="13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="V22" s="12">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="W22" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="X22" s="12">
-        <v>1637</v>
+        <v>1670</v>
       </c>
       <c r="Y22" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="Z22" s="12">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="AA22" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AB22" s="12">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="AC22" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AD22" s="12">
-        <v>24396</v>
+        <v>25193</v>
       </c>
       <c r="AE22" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AF22" s="12">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="AG22" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AH22" s="12">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AI22" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AJ22" s="12">
-        <v>9441</v>
+        <v>9655</v>
       </c>
       <c r="AK22" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AL22" s="12">
         <v>4070</v>
       </c>
       <c r="AM22" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AN22" s="12">
         <v>4</v>
@@ -4139,7 +4166,7 @@
         <v>26</v>
       </c>
       <c r="AS22" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 31/08/2026  8:57:50,55
</commit_message>
<xml_diff>
--- a/data/20260823_125317_Radar_Anomali_Keluarga_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Kabupaten_Kota.xlsx
+++ b/data/20260823_125317_Radar_Anomali_Keluarga_Anomali_1_Anomali_2_Anomali_3_Anomali_4_Anomali_5_Anomali_6_Anomali_7_Kabupaten_Kota.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="303">
   <si>
     <t>DATA RADAR ANOMALI KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 29 Agu 2026, 16.20</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Dicetak: 31 Agu 2026, 08.57</t>
   </si>
   <si>
     <t>Kode</t>
@@ -298,631 +298,622 @@
     <t>0,01</t>
   </si>
   <si>
-    <t>4,19</t>
+    <t>4,21</t>
+  </si>
+  <si>
+    <t>0,66</t>
+  </si>
+  <si>
+    <t>20,04</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>0,32</t>
   </si>
   <si>
     <t>0,68</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>19,66</t>
+    <t>2,4</t>
+  </si>
+  <si>
+    <t>0,19</t>
+  </si>
+  <si>
+    <t>2,89</t>
+  </si>
+  <si>
+    <t>0,54</t>
+  </si>
+  <si>
+    <t>43,37</t>
+  </si>
+  <si>
+    <t>1,01</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>16,52</t>
+  </si>
+  <si>
+    <t>6,77</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>3,76</t>
+  </si>
+  <si>
+    <t>0,82</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>27,88</t>
+  </si>
+  <si>
+    <t>0,59</t>
+  </si>
+  <si>
+    <t>1,11</t>
+  </si>
+  <si>
+    <t>4,07</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>38,2</t>
+  </si>
+  <si>
+    <t>0,44</t>
+  </si>
+  <si>
+    <t>12,84</t>
+  </si>
+  <si>
+    <t>9,78</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>6,55</t>
+  </si>
+  <si>
+    <t>19,76</t>
+  </si>
+  <si>
+    <t>0,3</t>
+  </si>
+  <si>
+    <t>0,9</t>
+  </si>
+  <si>
+    <t>3,3</t>
+  </si>
+  <si>
+    <t>0,18</t>
+  </si>
+  <si>
+    <t>3,18</t>
+  </si>
+  <si>
+    <t>41,8</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>22,7</t>
+  </si>
+  <si>
+    <t>0,42</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>5,81</t>
+  </si>
+  <si>
+    <t>0,37</t>
+  </si>
+  <si>
+    <t>19,03</t>
+  </si>
+  <si>
+    <t>0,56</t>
+  </si>
+  <si>
+    <t>3,25</t>
+  </si>
+  <si>
+    <t>3,35</t>
+  </si>
+  <si>
+    <t>0,74</t>
+  </si>
+  <si>
+    <t>43,83</t>
+  </si>
+  <si>
+    <t>3,96</t>
+  </si>
+  <si>
+    <t>17,86</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>4,33</t>
   </si>
   <si>
     <t>0,36</t>
   </si>
   <si>
-    <t>0,69</t>
+    <t>25,02</t>
+  </si>
+  <si>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>1,1</t>
+  </si>
+  <si>
+    <t>2,64</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>0,33</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>43,14</t>
+  </si>
+  <si>
+    <t>0,4</t>
+  </si>
+  <si>
+    <t>15,23</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>22,03</t>
+  </si>
+  <si>
+    <t>0,45</t>
+  </si>
+  <si>
+    <t>5,83</t>
+  </si>
+  <si>
+    <t>4,18</t>
+  </si>
+  <si>
+    <t>0,47</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>44,89</t>
+  </si>
+  <si>
+    <t>1,18</t>
+  </si>
+  <si>
+    <t>15,16</t>
+  </si>
+  <si>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>2,57</t>
+  </si>
+  <si>
+    <t>2,3</t>
+  </si>
+  <si>
+    <t>14,37</t>
+  </si>
+  <si>
+    <t>0,05</t>
+  </si>
+  <si>
+    <t>2,25</t>
   </si>
   <si>
     <t>2,44</t>
   </si>
   <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>2,87</t>
-  </si>
-  <si>
     <t>0,55</t>
   </si>
   <si>
-    <t>0,33</t>
-  </si>
-  <si>
-    <t>43,28</t>
-  </si>
-  <si>
-    <t>1,04</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>16,58</t>
-  </si>
-  <si>
-    <t>6,99</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>3,82</t>
-  </si>
-  <si>
-    <t>0,97</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>25,85</t>
-  </si>
-  <si>
-    <t>0,7</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>1,52</t>
-  </si>
-  <si>
-    <t>4,09</t>
+    <t>44,41</t>
+  </si>
+  <si>
+    <t>0,78</t>
+  </si>
+  <si>
+    <t>16,77</t>
+  </si>
+  <si>
+    <t>12,9</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>4,36</t>
+  </si>
+  <si>
+    <t>20,1</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>38,27</t>
-  </si>
-  <si>
-    <t>0,52</t>
-  </si>
-  <si>
-    <t>12,27</t>
-  </si>
-  <si>
-    <t>11,52</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>6,55</t>
-  </si>
-  <si>
-    <t>19,78</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>0,9</t>
+    <t>2,49</t>
+  </si>
+  <si>
+    <t>2,96</t>
+  </si>
+  <si>
+    <t>41,29</t>
+  </si>
+  <si>
+    <t>0,34</t>
+  </si>
+  <si>
+    <t>26,01</t>
+  </si>
+  <si>
+    <t>1,21</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>4,47</t>
+  </si>
+  <si>
+    <t>21,51</t>
+  </si>
+  <si>
+    <t>0,91</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>2,15</t>
+  </si>
+  <si>
+    <t>0,46</t>
+  </si>
+  <si>
+    <t>2,01</t>
+  </si>
+  <si>
+    <t>46,21</t>
+  </si>
+  <si>
+    <t>15,53</t>
+  </si>
+  <si>
+    <t>4,52</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>13,41</t>
+  </si>
+  <si>
+    <t>0,35</t>
+  </si>
+  <si>
+    <t>0,96</t>
+  </si>
+  <si>
+    <t>1,17</t>
+  </si>
+  <si>
+    <t>1,27</t>
+  </si>
+  <si>
+    <t>40,65</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>14,7</t>
+  </si>
+  <si>
+    <t>22,02</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>5,02</t>
+  </si>
+  <si>
+    <t>15,4</t>
+  </si>
+  <si>
+    <t>0,64</t>
+  </si>
+  <si>
+    <t>1,38</t>
+  </si>
+  <si>
+    <t>4,97</t>
+  </si>
+  <si>
+    <t>4,08</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>0,89</t>
+  </si>
+  <si>
+    <t>42,84</t>
+  </si>
+  <si>
+    <t>1,57</t>
+  </si>
+  <si>
+    <t>18,94</t>
+  </si>
+  <si>
+    <t>2,75</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>4,46</t>
+  </si>
+  <si>
+    <t>0,75</t>
+  </si>
+  <si>
+    <t>21,26</t>
+  </si>
+  <si>
+    <t>0,84</t>
+  </si>
+  <si>
+    <t>0,87</t>
+  </si>
+  <si>
+    <t>1,65</t>
+  </si>
+  <si>
+    <t>49,54</t>
+  </si>
+  <si>
+    <t>1,22</t>
+  </si>
+  <si>
+    <t>11,94</t>
+  </si>
+  <si>
+    <t>6,37</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>0,14</t>
+  </si>
+  <si>
+    <t>20,89</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>1,83</t>
+  </si>
+  <si>
+    <t>45,59</t>
+  </si>
+  <si>
+    <t>0,28</t>
+  </si>
+  <si>
+    <t>22,95</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>4,56</t>
+  </si>
+  <si>
+    <t>26,78</t>
+  </si>
+  <si>
+    <t>0,38</t>
   </si>
   <si>
     <t>3,31</t>
   </si>
   <si>
-    <t>0,18</t>
-  </si>
-  <si>
-    <t>3,19</t>
-  </si>
-  <si>
-    <t>0,3</t>
-  </si>
-  <si>
-    <t>41,85</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>22,73</t>
-  </si>
-  <si>
-    <t>0,42</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>5,81</t>
-  </si>
-  <si>
-    <t>0,37</t>
-  </si>
-  <si>
-    <t>19,03</t>
-  </si>
-  <si>
-    <t>0,56</t>
-  </si>
-  <si>
-    <t>3,25</t>
-  </si>
-  <si>
-    <t>3,35</t>
-  </si>
-  <si>
-    <t>0,74</t>
-  </si>
-  <si>
-    <t>43,81</t>
-  </si>
-  <si>
-    <t>3,96</t>
-  </si>
-  <si>
-    <t>17,86</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>4,36</t>
-  </si>
-  <si>
-    <t>24,87</t>
-  </si>
-  <si>
-    <t>0,28</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>2,7</t>
-  </si>
-  <si>
-    <t>0,29</t>
-  </si>
-  <si>
-    <t>3,38</t>
-  </si>
-  <si>
-    <t>0,34</t>
-  </si>
-  <si>
-    <t>1,76</t>
-  </si>
-  <si>
-    <t>42,99</t>
+    <t>44,24</t>
+  </si>
+  <si>
+    <t>0,58</t>
+  </si>
+  <si>
+    <t>15,97</t>
+  </si>
+  <si>
+    <t>3,26</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>7,14</t>
+  </si>
+  <si>
+    <t>0,93</t>
+  </si>
+  <si>
+    <t>9,47</t>
+  </si>
+  <si>
+    <t>0,62</t>
+  </si>
+  <si>
+    <t>2,02</t>
+  </si>
+  <si>
+    <t>13,66</t>
+  </si>
+  <si>
+    <t>36,96</t>
+  </si>
+  <si>
+    <t>1,86</t>
+  </si>
+  <si>
+    <t>9,32</t>
+  </si>
+  <si>
+    <t>2,95</t>
+  </si>
+  <si>
+    <t>0,31</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>2,45</t>
   </si>
   <si>
     <t>0,41</t>
   </si>
   <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>15,19</t>
-  </si>
-  <si>
-    <t>1,73</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>4,2</t>
-  </si>
-  <si>
-    <t>22,04</t>
-  </si>
-  <si>
-    <t>0,45</t>
-  </si>
-  <si>
-    <t>5,84</t>
-  </si>
-  <si>
-    <t>0,47</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>44,87</t>
-  </si>
-  <si>
-    <t>1,18</t>
-  </si>
-  <si>
-    <t>15,18</t>
-  </si>
-  <si>
-    <t>0,63</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>2,58</t>
-  </si>
-  <si>
-    <t>2,3</t>
-  </si>
-  <si>
-    <t>14,39</t>
-  </si>
-  <si>
-    <t>0,05</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>2,25</t>
-  </si>
-  <si>
-    <t>44,38</t>
-  </si>
-  <si>
-    <t>0,79</t>
-  </si>
-  <si>
-    <t>16,75</t>
-  </si>
-  <si>
-    <t>12,92</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>4,33</t>
-  </si>
-  <si>
-    <t>20,04</t>
-  </si>
-  <si>
-    <t>0,13</t>
-  </si>
-  <si>
-    <t>0,6</t>
-  </si>
-  <si>
-    <t>2,48</t>
-  </si>
-  <si>
-    <t>2,95</t>
-  </si>
-  <si>
-    <t>0,38</t>
-  </si>
-  <si>
-    <t>41,25</t>
-  </si>
-  <si>
-    <t>0,31</t>
+    <t>11,56</t>
+  </si>
+  <si>
+    <t>0,61</t>
+  </si>
+  <si>
+    <t>2,38</t>
+  </si>
+  <si>
+    <t>2,52</t>
+  </si>
+  <si>
+    <t>2,65</t>
+  </si>
+  <si>
+    <t>1,02</t>
+  </si>
+  <si>
+    <t>41,88</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>8,09</t>
   </si>
   <si>
     <t>26,1</t>
-  </si>
-  <si>
-    <t>1,22</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>0,78</t>
-  </si>
-  <si>
-    <t>21,49</t>
-  </si>
-  <si>
-    <t>0,92</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>2,16</t>
-  </si>
-  <si>
-    <t>0,46</t>
-  </si>
-  <si>
-    <t>2,02</t>
-  </si>
-  <si>
-    <t>46,37</t>
-  </si>
-  <si>
-    <t>15,43</t>
-  </si>
-  <si>
-    <t>4,55</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>3,29</t>
-  </si>
-  <si>
-    <t>13,41</t>
-  </si>
-  <si>
-    <t>0,95</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>1,26</t>
-  </si>
-  <si>
-    <t>40,61</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>14,7</t>
-  </si>
-  <si>
-    <t>22,05</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>4,98</t>
-  </si>
-  <si>
-    <t>15,15</t>
-  </si>
-  <si>
-    <t>0,65</t>
-  </si>
-  <si>
-    <t>1,41</t>
-  </si>
-  <si>
-    <t>5,08</t>
-  </si>
-  <si>
-    <t>4,13</t>
-  </si>
-  <si>
-    <t>1,01</t>
-  </si>
-  <si>
-    <t>0,91</t>
-  </si>
-  <si>
-    <t>43,18</t>
-  </si>
-  <si>
-    <t>1,61</t>
-  </si>
-  <si>
-    <t>18,52</t>
-  </si>
-  <si>
-    <t>2,82</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>0,82</t>
-  </si>
-  <si>
-    <t>20,42</t>
-  </si>
-  <si>
-    <t>0,73</t>
-  </si>
-  <si>
-    <t>0,89</t>
-  </si>
-  <si>
-    <t>1,55</t>
-  </si>
-  <si>
-    <t>49,04</t>
-  </si>
-  <si>
-    <t>1,33</t>
-  </si>
-  <si>
-    <t>12,46</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>4,15</t>
-  </si>
-  <si>
-    <t>0,14</t>
-  </si>
-  <si>
-    <t>20,71</t>
-  </si>
-  <si>
-    <t>0,51</t>
-  </si>
-  <si>
-    <t>0,48</t>
-  </si>
-  <si>
-    <t>1,62</t>
-  </si>
-  <si>
-    <t>0,17</t>
-  </si>
-  <si>
-    <t>1,64</t>
-  </si>
-  <si>
-    <t>45,67</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>23,03</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>4,45</t>
-  </si>
-  <si>
-    <t>26,53</t>
-  </si>
-  <si>
-    <t>0,43</t>
-  </si>
-  <si>
-    <t>3,34</t>
-  </si>
-  <si>
-    <t>43,25</t>
-  </si>
-  <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>16,62</t>
-  </si>
-  <si>
-    <t>3,69</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>6,96</t>
-  </si>
-  <si>
-    <t>9,18</t>
-  </si>
-  <si>
-    <t>6,49</t>
-  </si>
-  <si>
-    <t>2,53</t>
-  </si>
-  <si>
-    <t>7,28</t>
-  </si>
-  <si>
-    <t>13,92</t>
-  </si>
-  <si>
-    <t>36,55</t>
-  </si>
-  <si>
-    <t>1,9</t>
-  </si>
-  <si>
-    <t>9,02</t>
-  </si>
-  <si>
-    <t>3,01</t>
-  </si>
-  <si>
-    <t>0,32</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>2,45</t>
-  </si>
-  <si>
-    <t>11,56</t>
-  </si>
-  <si>
-    <t>0,61</t>
-  </si>
-  <si>
-    <t>2,38</t>
-  </si>
-  <si>
-    <t>2,52</t>
-  </si>
-  <si>
-    <t>2,65</t>
-  </si>
-  <si>
-    <t>1,09</t>
-  </si>
-  <si>
-    <t>41,84</t>
-  </si>
-  <si>
-    <t>0,2</t>
-  </si>
-  <si>
-    <t>8,1</t>
-  </si>
-  <si>
-    <t>26,12</t>
   </si>
   <si>
     <t/>
@@ -1848,7 +1839,7 @@
         <v>93</v>
       </c>
       <c r="C6" s="6">
-        <v>58216</v>
+        <v>60113</v>
       </c>
       <c r="D6" s="6">
         <v>7</v>
@@ -1857,7 +1848,7 @@
         <v>94</v>
       </c>
       <c r="F6" s="6">
-        <v>2441</v>
+        <v>2528</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>95</v>
@@ -1869,94 +1860,94 @@
         <v>96</v>
       </c>
       <c r="J6" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="L6" s="6">
+        <v>12044</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>97</v>
-      </c>
-      <c r="L6" s="6">
-        <v>11446</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>98</v>
       </c>
       <c r="N6" s="6">
         <v>3</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="P6" s="6">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="Q6" s="7" t="s">
         <v>99</v>
       </c>
       <c r="R6" s="6">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>100</v>
       </c>
       <c r="T6" s="6">
-        <v>1423</v>
+        <v>1443</v>
       </c>
       <c r="U6" s="7" t="s">
         <v>101</v>
       </c>
       <c r="V6" s="6">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="W6" s="7" t="s">
         <v>102</v>
       </c>
       <c r="X6" s="6">
-        <v>1670</v>
+        <v>1735</v>
       </c>
       <c r="Y6" s="7" t="s">
         <v>103</v>
       </c>
       <c r="Z6" s="6">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="AA6" s="7" t="s">
         <v>104</v>
       </c>
       <c r="AB6" s="6">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AC6" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="AD6" s="6">
+        <v>26070</v>
+      </c>
+      <c r="AE6" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="AD6" s="6">
-        <v>25193</v>
-      </c>
-      <c r="AE6" s="7" t="s">
+      <c r="AF6" s="6">
+        <v>607</v>
+      </c>
+      <c r="AG6" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="AF6" s="6">
-        <v>603</v>
-      </c>
-      <c r="AG6" s="7" t="s">
+      <c r="AH6" s="6">
+        <v>12</v>
+      </c>
+      <c r="AI6" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="AH6" s="6">
-        <v>14</v>
-      </c>
-      <c r="AI6" s="7" t="s">
+      <c r="AJ6" s="6">
+        <v>9930</v>
+      </c>
+      <c r="AK6" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="AJ6" s="6">
-        <v>9655</v>
-      </c>
-      <c r="AK6" s="7" t="s">
+      <c r="AL6" s="6">
+        <v>4072</v>
+      </c>
+      <c r="AM6" s="7" t="s">
         <v>109</v>
-      </c>
-      <c r="AL6" s="6">
-        <v>4070</v>
-      </c>
-      <c r="AM6" s="7" t="s">
-        <v>110</v>
       </c>
       <c r="AN6" s="6">
         <v>4</v>
@@ -1968,295 +1959,295 @@
         <v>0</v>
       </c>
       <c r="AQ6" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR6" s="6">
         <v>26</v>
       </c>
       <c r="AS6" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="9">
+        <v>3885</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="9">
+        <v>146</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="C7" s="9">
-        <v>3300</v>
-      </c>
-      <c r="D7" s="9">
-        <v>0</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="F7" s="9">
-        <v>126</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>114</v>
       </c>
       <c r="H7" s="9">
         <v>32</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="J7" s="9">
+        <v>4</v>
+      </c>
+      <c r="K7" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="J7" s="9">
-        <v>1</v>
-      </c>
-      <c r="K7" s="10" t="s">
+      <c r="L7" s="9">
+        <v>1083</v>
+      </c>
+      <c r="M7" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="L7" s="9">
-        <v>853</v>
-      </c>
-      <c r="M7" s="10" t="s">
-        <v>117</v>
-      </c>
       <c r="N7" s="9">
         <v>0</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P7" s="9">
         <v>23</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R7" s="9">
         <v>4</v>
       </c>
       <c r="S7" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="T7" s="9">
         <v>4</v>
       </c>
       <c r="U7" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="V7" s="9">
+        <v>43</v>
+      </c>
+      <c r="W7" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="X7" s="9">
+        <v>158</v>
+      </c>
+      <c r="Y7" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="V7" s="9">
-        <v>50</v>
-      </c>
-      <c r="W7" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="X7" s="9">
-        <v>135</v>
-      </c>
-      <c r="Y7" s="10" t="s">
-        <v>121</v>
       </c>
       <c r="Z7" s="9">
         <v>3</v>
       </c>
       <c r="AA7" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="AB7" s="9">
+        <v>5</v>
+      </c>
+      <c r="AC7" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="AD7" s="9">
+        <v>1484</v>
+      </c>
+      <c r="AE7" s="10" t="s">
         <v>122</v>
-      </c>
-      <c r="AB7" s="9">
-        <v>4</v>
-      </c>
-      <c r="AC7" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="AD7" s="9">
-        <v>1263</v>
-      </c>
-      <c r="AE7" s="10" t="s">
-        <v>123</v>
       </c>
       <c r="AF7" s="9">
         <v>17</v>
       </c>
       <c r="AG7" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH7" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI7" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ7" s="9">
+        <v>499</v>
+      </c>
+      <c r="AK7" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="AH7" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI7" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="AJ7" s="9">
-        <v>405</v>
-      </c>
-      <c r="AK7" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="AL7" s="9">
         <v>380</v>
       </c>
       <c r="AM7" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AN7" s="9">
         <v>0</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP7" s="9">
         <v>0</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR7" s="9">
         <v>0</v>
       </c>
       <c r="AS7" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>128</v>
-      </c>
       <c r="C8" s="9">
-        <v>1663</v>
+        <v>1665</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F8" s="9">
         <v>109</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H8" s="9">
         <v>0</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J8" s="9">
         <v>0</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L8" s="9">
         <v>329</v>
       </c>
       <c r="M8" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="N8" s="9">
+        <v>0</v>
+      </c>
+      <c r="O8" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="P8" s="9">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="N8" s="9">
-        <v>0</v>
-      </c>
-      <c r="O8" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="P8" s="9">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="R8" s="9">
         <v>15</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="T8" s="9">
         <v>55</v>
       </c>
       <c r="U8" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="V8" s="9">
         <v>3</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="X8" s="9">
         <v>53</v>
       </c>
       <c r="Y8" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Z8" s="9">
         <v>5</v>
       </c>
       <c r="AA8" s="10" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="AB8" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC8" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AD8" s="9">
         <v>696</v>
       </c>
       <c r="AE8" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AF8" s="9">
         <v>2</v>
       </c>
       <c r="AG8" s="10" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="AH8" s="9">
         <v>1</v>
       </c>
       <c r="AI8" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AJ8" s="9">
         <v>378</v>
       </c>
       <c r="AK8" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AL8" s="9">
         <v>7</v>
       </c>
       <c r="AM8" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AN8" s="9">
         <v>0</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP8" s="9">
         <v>0</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR8" s="9">
         <v>2</v>
       </c>
       <c r="AS8" s="10" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>141</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>142</v>
       </c>
       <c r="C9" s="9">
         <v>5939</v>
@@ -2265,165 +2256,165 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F9" s="9">
         <v>345</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H9" s="9">
         <v>22</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J9" s="9">
         <v>0</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L9" s="9">
         <v>1130</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N9" s="9">
         <v>0</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P9" s="9">
         <v>0</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="R9" s="9">
         <v>33</v>
       </c>
       <c r="S9" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="T9" s="9">
         <v>193</v>
       </c>
       <c r="U9" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="V9" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W9" s="10" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="X9" s="9">
         <v>199</v>
       </c>
       <c r="Y9" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="Z9" s="9">
         <v>44</v>
       </c>
       <c r="AA9" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="AD9" s="9">
+        <v>2603</v>
+      </c>
+      <c r="AE9" s="10" t="s">
         <v>149</v>
-      </c>
-      <c r="AB9" s="9">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="AD9" s="9">
-        <v>2602</v>
-      </c>
-      <c r="AE9" s="10" t="s">
-        <v>150</v>
       </c>
       <c r="AF9" s="9">
         <v>235</v>
       </c>
       <c r="AG9" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AH9" s="9">
         <v>0</v>
       </c>
       <c r="AI9" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ9" s="9">
         <v>1061</v>
       </c>
       <c r="AK9" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="AL9" s="9">
         <v>68</v>
       </c>
       <c r="AM9" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AN9" s="9">
         <v>0</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP9" s="9">
         <v>0</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR9" s="9">
         <v>4</v>
       </c>
       <c r="AS9" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>156</v>
-      </c>
       <c r="C10" s="9">
-        <v>6859</v>
+        <v>7017</v>
       </c>
       <c r="D10" s="9">
         <v>3</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F10" s="9">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H10" s="9">
         <v>25</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>99</v>
+        <v>157</v>
       </c>
       <c r="J10" s="9">
         <v>0</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L10" s="9">
-        <v>1706</v>
+        <v>1756</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>158</v>
@@ -2441,7 +2432,7 @@
         <v>159</v>
       </c>
       <c r="R10" s="9">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>160</v>
@@ -2453,58 +2444,58 @@
         <v>161</v>
       </c>
       <c r="V10" s="9">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="W10" s="10" t="s">
         <v>162</v>
       </c>
       <c r="X10" s="9">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="Y10" s="10" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="Z10" s="9">
         <v>23</v>
       </c>
       <c r="AA10" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="AB10" s="9">
+        <v>119</v>
+      </c>
+      <c r="AC10" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="AB10" s="9">
-        <v>121</v>
-      </c>
-      <c r="AC10" s="10" t="s">
+      <c r="AD10" s="9">
+        <v>3027</v>
+      </c>
+      <c r="AE10" s="10" t="s">
         <v>165</v>
-      </c>
-      <c r="AD10" s="9">
-        <v>2949</v>
-      </c>
-      <c r="AE10" s="10" t="s">
-        <v>166</v>
       </c>
       <c r="AF10" s="9">
         <v>28</v>
       </c>
       <c r="AG10" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="AH10" s="9">
+        <v>5</v>
+      </c>
+      <c r="AI10" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="AJ10" s="9">
+        <v>1069</v>
+      </c>
+      <c r="AK10" s="10" t="s">
         <v>167</v>
-      </c>
-      <c r="AH10" s="9">
-        <v>7</v>
-      </c>
-      <c r="AI10" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="AJ10" s="9">
-        <v>1042</v>
-      </c>
-      <c r="AK10" s="10" t="s">
-        <v>169</v>
       </c>
       <c r="AL10" s="9">
         <v>119</v>
       </c>
       <c r="AM10" s="10" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="AN10" s="9">
         <v>1</v>
@@ -2516,680 +2507,680 @@
         <v>0</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR10" s="9">
         <v>3</v>
       </c>
       <c r="AS10" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C11" s="9">
-        <v>6185</v>
+        <v>6195</v>
       </c>
       <c r="D11" s="9">
         <v>2</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="F11" s="9">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>173</v>
+        <v>95</v>
       </c>
       <c r="H11" s="9">
         <v>6</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
       <c r="J11" s="9">
         <v>0</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L11" s="9">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="N11" s="9">
         <v>0</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P11" s="9">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>104</v>
+        <v>145</v>
       </c>
       <c r="R11" s="9">
         <v>28</v>
       </c>
       <c r="S11" s="10" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="T11" s="9">
         <v>361</v>
       </c>
       <c r="U11" s="10" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="V11" s="9">
         <v>6</v>
       </c>
       <c r="W11" s="10" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
       <c r="X11" s="9">
         <v>259</v>
       </c>
       <c r="Y11" s="10" t="s">
-        <v>95</v>
+        <v>174</v>
       </c>
       <c r="Z11" s="9">
         <v>29</v>
       </c>
       <c r="AA11" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AB11" s="9">
         <v>9</v>
       </c>
       <c r="AC11" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AD11" s="9">
-        <v>2775</v>
+        <v>2781</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="AF11" s="9">
         <v>73</v>
       </c>
       <c r="AG11" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="AH11" s="9">
         <v>0</v>
       </c>
       <c r="AI11" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ11" s="9">
         <v>939</v>
       </c>
       <c r="AK11" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="AL11" s="9">
         <v>39</v>
       </c>
       <c r="AM11" s="10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AN11" s="9">
         <v>0</v>
       </c>
       <c r="AO11" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP11" s="9">
         <v>0</v>
       </c>
       <c r="AQ11" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR11" s="9">
         <v>2</v>
       </c>
       <c r="AS11" s="10" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C12" s="9">
-        <v>5858</v>
+        <v>5866</v>
       </c>
       <c r="D12" s="9">
         <v>0</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F12" s="9">
         <v>151</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H12" s="9">
         <v>135</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="J12" s="9">
         <v>0</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L12" s="9">
         <v>843</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="N12" s="9">
         <v>0</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P12" s="9">
         <v>3</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="R12" s="9">
         <v>26</v>
       </c>
       <c r="S12" s="10" t="s">
-        <v>189</v>
+        <v>123</v>
       </c>
       <c r="T12" s="9">
         <v>132</v>
       </c>
       <c r="U12" s="10" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="V12" s="9">
         <v>2</v>
       </c>
       <c r="W12" s="10" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="X12" s="9">
         <v>143</v>
       </c>
       <c r="Y12" s="10" t="s">
-        <v>101</v>
+        <v>188</v>
       </c>
       <c r="Z12" s="9">
         <v>32</v>
       </c>
       <c r="AA12" s="10" t="s">
-        <v>104</v>
+        <v>189</v>
       </c>
       <c r="AB12" s="9">
         <v>0</v>
       </c>
       <c r="AC12" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AD12" s="9">
-        <v>2600</v>
+        <v>2605</v>
       </c>
       <c r="AE12" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AF12" s="9">
         <v>46</v>
       </c>
       <c r="AG12" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="AH12" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ12" s="9">
+        <v>984</v>
+      </c>
+      <c r="AK12" s="10" t="s">
         <v>192</v>
-      </c>
-      <c r="AH12" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="AJ12" s="9">
-        <v>981</v>
-      </c>
-      <c r="AK12" s="10" t="s">
-        <v>193</v>
       </c>
       <c r="AL12" s="9">
         <v>757</v>
       </c>
       <c r="AM12" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AN12" s="9">
         <v>1</v>
       </c>
       <c r="AO12" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AP12" s="9">
         <v>0</v>
       </c>
       <c r="AQ12" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR12" s="9">
         <v>6</v>
       </c>
       <c r="AS12" s="10" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="C13" s="9">
+        <v>3214</v>
+      </c>
+      <c r="D13" s="9">
+        <v>0</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="9">
+        <v>140</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>196</v>
-      </c>
-      <c r="C13" s="9">
-        <v>3188</v>
-      </c>
-      <c r="D13" s="9">
-        <v>0</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" s="9">
-        <v>138</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>197</v>
       </c>
       <c r="H13" s="9">
         <v>2</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J13" s="9">
         <v>0</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L13" s="9">
-        <v>639</v>
+        <v>646</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="N13" s="9">
         <v>1</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="P13" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="R13" s="9">
         <v>19</v>
       </c>
       <c r="S13" s="10" t="s">
-        <v>200</v>
+        <v>117</v>
       </c>
       <c r="T13" s="9">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U13" s="10" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="V13" s="9">
         <v>3</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>122</v>
+        <v>198</v>
       </c>
       <c r="X13" s="9">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Y13" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="Z13" s="9">
         <v>12</v>
       </c>
       <c r="AA13" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="AB13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="AD13" s="9">
+        <v>1327</v>
+      </c>
+      <c r="AE13" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF13" s="9">
+        <v>11</v>
+      </c>
+      <c r="AG13" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="AH13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AI13" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ13" s="9">
+        <v>836</v>
+      </c>
+      <c r="AK13" s="10" t="s">
         <v>203</v>
-      </c>
-      <c r="AB13" s="9">
-        <v>1</v>
-      </c>
-      <c r="AC13" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AD13" s="9">
-        <v>1315</v>
-      </c>
-      <c r="AE13" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="AF13" s="9">
-        <v>10</v>
-      </c>
-      <c r="AG13" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="AH13" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="AJ13" s="9">
-        <v>832</v>
-      </c>
-      <c r="AK13" s="10" t="s">
-        <v>206</v>
       </c>
       <c r="AL13" s="9">
         <v>39</v>
       </c>
       <c r="AM13" s="10" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="AN13" s="9">
         <v>0</v>
       </c>
       <c r="AO13" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP13" s="9">
         <v>0</v>
       </c>
       <c r="AQ13" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR13" s="9">
         <v>0</v>
       </c>
       <c r="AS13" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C14" s="9">
-        <v>2178</v>
+        <v>2190</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F14" s="9">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>157</v>
+        <v>207</v>
       </c>
       <c r="H14" s="9">
         <v>17</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>210</v>
+        <v>191</v>
       </c>
       <c r="J14" s="9">
         <v>0</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L14" s="9">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="N14" s="9">
         <v>1</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="P14" s="9">
         <v>20</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="R14" s="9">
         <v>26</v>
       </c>
       <c r="S14" s="10" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="T14" s="9">
         <v>47</v>
       </c>
       <c r="U14" s="10" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="V14" s="9">
         <v>10</v>
       </c>
       <c r="W14" s="10" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="X14" s="9">
         <v>44</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="Z14" s="9">
         <v>1</v>
       </c>
       <c r="AA14" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AB14" s="9">
         <v>0</v>
       </c>
       <c r="AC14" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AD14" s="9">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="AE14" s="10" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="AF14" s="9">
         <v>2</v>
       </c>
       <c r="AG14" s="10" t="s">
-        <v>122</v>
+        <v>198</v>
       </c>
       <c r="AH14" s="9">
         <v>0</v>
       </c>
       <c r="AI14" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ14" s="9">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="AK14" s="10" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AL14" s="9">
         <v>99</v>
       </c>
       <c r="AM14" s="10" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="AN14" s="9">
         <v>1</v>
       </c>
       <c r="AO14" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AP14" s="9">
         <v>0</v>
       </c>
       <c r="AQ14" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR14" s="9">
         <v>1</v>
       </c>
       <c r="AS14" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C15" s="9">
-        <v>7693</v>
+        <v>7703</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F15" s="9">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="H15" s="9">
         <v>88</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J15" s="9">
         <v>0</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L15" s="9">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="M15" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="N15" s="9">
+        <v>0</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="P15" s="9">
+        <v>27</v>
+      </c>
+      <c r="Q15" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="R15" s="9">
+        <v>74</v>
+      </c>
+      <c r="S15" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="T15" s="9">
+        <v>90</v>
+      </c>
+      <c r="U15" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="V15" s="9">
+        <v>2</v>
+      </c>
+      <c r="W15" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="X15" s="9">
+        <v>98</v>
+      </c>
+      <c r="Y15" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="N15" s="9">
-        <v>0</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="P15" s="9">
-        <v>42</v>
-      </c>
-      <c r="Q15" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="R15" s="9">
-        <v>73</v>
-      </c>
-      <c r="S15" s="10" t="s">
+      <c r="Z15" s="9">
+        <v>9</v>
+      </c>
+      <c r="AA15" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB15" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="AD15" s="9">
+        <v>3131</v>
+      </c>
+      <c r="AE15" s="10" t="s">
         <v>224</v>
-      </c>
-      <c r="T15" s="9">
-        <v>76</v>
-      </c>
-      <c r="U15" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="V15" s="9">
-        <v>4</v>
-      </c>
-      <c r="W15" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="X15" s="9">
-        <v>97</v>
-      </c>
-      <c r="Y15" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="Z15" s="9">
-        <v>8</v>
-      </c>
-      <c r="AA15" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="AB15" s="9">
-        <v>0</v>
-      </c>
-      <c r="AC15" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="AD15" s="9">
-        <v>3124</v>
-      </c>
-      <c r="AE15" s="10" t="s">
-        <v>227</v>
       </c>
       <c r="AF15" s="9">
         <v>66</v>
       </c>
       <c r="AG15" s="10" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="AH15" s="9">
         <v>0</v>
       </c>
       <c r="AI15" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ15" s="9">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="AL15" s="9">
         <v>1696</v>
       </c>
       <c r="AM15" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="AN15" s="9">
         <v>1</v>
@@ -3201,846 +3192,846 @@
         <v>0</v>
       </c>
       <c r="AQ15" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR15" s="9">
         <v>2</v>
       </c>
       <c r="AS15" s="10" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C16" s="9">
-        <v>1987</v>
+        <v>2033</v>
       </c>
       <c r="D16" s="9">
         <v>0</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F16" s="9">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="H16" s="9">
         <v>6</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="J16" s="9">
         <v>0</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L16" s="9">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="N16" s="9">
         <v>0</v>
       </c>
       <c r="O16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P16" s="9">
         <v>13</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="R16" s="9">
         <v>28</v>
       </c>
       <c r="S16" s="10" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="T16" s="9">
         <v>101</v>
       </c>
       <c r="U16" s="10" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="V16" s="9">
         <v>0</v>
       </c>
       <c r="W16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="X16" s="9">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Y16" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="Z16" s="9">
         <v>20</v>
       </c>
       <c r="AA16" s="10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="AB16" s="9">
         <v>18</v>
       </c>
       <c r="AC16" s="10" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="AD16" s="9">
-        <v>858</v>
+        <v>871</v>
       </c>
       <c r="AE16" s="10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="AF16" s="9">
         <v>32</v>
       </c>
       <c r="AG16" s="10" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="AH16" s="9">
         <v>3</v>
       </c>
       <c r="AI16" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AJ16" s="9">
-        <v>368</v>
+        <v>385</v>
       </c>
       <c r="AK16" s="10" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="AL16" s="9">
         <v>56</v>
       </c>
       <c r="AM16" s="10" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="AN16" s="9">
         <v>0</v>
       </c>
       <c r="AO16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP16" s="9">
         <v>0</v>
       </c>
       <c r="AQ16" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR16" s="9">
         <v>2</v>
       </c>
       <c r="AS16" s="10" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C17" s="9">
-        <v>3163</v>
+        <v>3452</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>116</v>
+        <v>170</v>
       </c>
       <c r="F17" s="9">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>157</v>
+        <v>244</v>
       </c>
       <c r="H17" s="9">
         <v>26</v>
       </c>
       <c r="I17" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="J17" s="9">
+        <v>0</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="L17" s="9">
+        <v>734</v>
+      </c>
+      <c r="M17" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="N17" s="9">
+        <v>0</v>
+      </c>
+      <c r="O17" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="P17" s="9">
+        <v>22</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="R17" s="9">
+        <v>29</v>
+      </c>
+      <c r="S17" s="10" t="s">
         <v>247</v>
-      </c>
-      <c r="J17" s="9">
-        <v>0</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="L17" s="9">
-        <v>646</v>
-      </c>
-      <c r="M17" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="N17" s="9">
-        <v>0</v>
-      </c>
-      <c r="O17" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="P17" s="9">
-        <v>23</v>
-      </c>
-      <c r="Q17" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="R17" s="9">
-        <v>28</v>
-      </c>
-      <c r="S17" s="10" t="s">
-        <v>250</v>
       </c>
       <c r="T17" s="9">
         <v>30</v>
       </c>
       <c r="U17" s="10" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="V17" s="9">
         <v>9</v>
       </c>
       <c r="W17" s="10" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="X17" s="9">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="Y17" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="Z17" s="9">
         <v>2</v>
       </c>
       <c r="AA17" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AB17" s="9">
         <v>2</v>
       </c>
       <c r="AC17" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AD17" s="9">
-        <v>1551</v>
+        <v>1710</v>
       </c>
       <c r="AE17" s="10" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="AF17" s="9">
         <v>42</v>
       </c>
       <c r="AG17" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="AH17" s="9">
+        <v>2</v>
+      </c>
+      <c r="AI17" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="AJ17" s="9">
+        <v>412</v>
+      </c>
+      <c r="AK17" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="AL17" s="9">
+        <v>220</v>
+      </c>
+      <c r="AM17" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="AH17" s="9">
-        <v>1</v>
-      </c>
-      <c r="AI17" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AJ17" s="9">
-        <v>394</v>
-      </c>
-      <c r="AK17" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="AL17" s="9">
-        <v>221</v>
-      </c>
-      <c r="AM17" s="10" t="s">
-        <v>110</v>
-      </c>
       <c r="AN17" s="9">
         <v>0</v>
       </c>
       <c r="AO17" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP17" s="9">
         <v>0</v>
       </c>
       <c r="AQ17" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR17" s="9">
         <v>0</v>
       </c>
       <c r="AS17" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>256</v>
-      </c>
       <c r="C18" s="9">
-        <v>4143</v>
+        <v>4361</v>
       </c>
       <c r="D18" s="9">
         <v>0</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F18" s="9">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>257</v>
+        <v>235</v>
       </c>
       <c r="H18" s="9">
         <v>6</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="J18" s="9">
         <v>0</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L18" s="9">
-        <v>858</v>
+        <v>911</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="N18" s="9">
         <v>0</v>
       </c>
       <c r="O18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P18" s="9">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="Q18" s="10" t="s">
-        <v>260</v>
+        <v>143</v>
       </c>
       <c r="R18" s="9">
         <v>20</v>
       </c>
       <c r="S18" s="10" t="s">
-        <v>261</v>
+        <v>212</v>
       </c>
       <c r="T18" s="9">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="U18" s="10" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="V18" s="9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W18" s="10" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="X18" s="9">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="Y18" s="10" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="Z18" s="9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA18" s="10" t="s">
-        <v>205</v>
+        <v>99</v>
       </c>
       <c r="AB18" s="9">
         <v>15</v>
       </c>
       <c r="AC18" s="10" t="s">
-        <v>99</v>
+        <v>202</v>
       </c>
       <c r="AD18" s="9">
-        <v>1892</v>
+        <v>1988</v>
       </c>
       <c r="AE18" s="10" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="AF18" s="9">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="AG18" s="10" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="AH18" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI18" s="10" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="AJ18" s="9">
-        <v>954</v>
+        <v>1001</v>
       </c>
       <c r="AK18" s="10" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="AL18" s="9">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AM18" s="10" t="s">
-        <v>115</v>
+        <v>263</v>
       </c>
       <c r="AN18" s="9">
         <v>0</v>
       </c>
       <c r="AO18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP18" s="9">
         <v>0</v>
       </c>
       <c r="AQ18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR18" s="9">
         <v>0</v>
       </c>
       <c r="AS18" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C19" s="9">
-        <v>3958</v>
+        <v>4478</v>
       </c>
       <c r="D19" s="9">
         <v>0</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F19" s="9">
-        <v>176</v>
+        <v>204</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="H19" s="9">
         <v>18</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="J19" s="9">
         <v>0</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L19" s="9">
-        <v>1050</v>
+        <v>1199</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="N19" s="9">
         <v>0</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P19" s="9">
         <v>0</v>
       </c>
       <c r="Q19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="R19" s="9">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S19" s="10" t="s">
-        <v>203</v>
+        <v>157</v>
       </c>
       <c r="T19" s="9">
         <v>17</v>
       </c>
       <c r="U19" s="10" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="V19" s="9">
         <v>0</v>
       </c>
       <c r="W19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="X19" s="9">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="Y19" s="10" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="Z19" s="9">
         <v>4</v>
       </c>
       <c r="AA19" s="10" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="AB19" s="9">
         <v>1</v>
       </c>
       <c r="AC19" s="10" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="AD19" s="9">
-        <v>1712</v>
+        <v>1981</v>
       </c>
       <c r="AE19" s="10" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="AF19" s="9">
         <v>26</v>
       </c>
       <c r="AG19" s="10" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="AH19" s="9">
         <v>1</v>
       </c>
       <c r="AI19" s="10" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="AJ19" s="9">
-        <v>658</v>
+        <v>715</v>
       </c>
       <c r="AK19" s="10" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="AL19" s="9">
         <v>146</v>
       </c>
       <c r="AM19" s="10" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="AN19" s="9">
         <v>0</v>
       </c>
       <c r="AO19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP19" s="9">
         <v>0</v>
       </c>
       <c r="AQ19" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR19" s="9">
         <v>2</v>
       </c>
       <c r="AS19" s="10" t="s">
-        <v>188</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C20" s="9">
-        <v>632</v>
+        <v>644</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F20" s="9">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="H20" s="9">
         <v>6</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>224</v>
+        <v>277</v>
       </c>
       <c r="J20" s="9">
         <v>0</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L20" s="9">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="N20" s="9">
         <v>0</v>
       </c>
       <c r="O20" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P20" s="9">
         <v>5</v>
       </c>
       <c r="Q20" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="R20" s="9">
         <v>4</v>
       </c>
       <c r="S20" s="10" t="s">
-        <v>182</v>
+        <v>279</v>
       </c>
       <c r="T20" s="9">
         <v>41</v>
       </c>
       <c r="U20" s="10" t="s">
-        <v>282</v>
+        <v>253</v>
       </c>
       <c r="V20" s="9">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="W20" s="10" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="X20" s="9">
         <v>46</v>
       </c>
       <c r="Y20" s="10" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="Z20" s="9">
         <v>88</v>
       </c>
       <c r="AA20" s="10" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="AB20" s="9">
         <v>3</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="AD20" s="9">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="AE20" s="10" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="AF20" s="9">
         <v>12</v>
       </c>
       <c r="AG20" s="10" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="AH20" s="9">
         <v>0</v>
       </c>
       <c r="AI20" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ20" s="9">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AK20" s="10" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="AL20" s="9">
         <v>19</v>
       </c>
       <c r="AM20" s="10" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="AN20" s="9">
         <v>0</v>
       </c>
       <c r="AO20" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP20" s="9">
         <v>0</v>
       </c>
       <c r="AQ20" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR20" s="9">
         <v>2</v>
       </c>
       <c r="AS20" s="10" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="C21" s="9">
-        <v>1470</v>
+        <v>1471</v>
       </c>
       <c r="D21" s="9">
         <v>0</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F21" s="9">
         <v>36</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="H21" s="9">
         <v>6</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>167</v>
+        <v>290</v>
       </c>
       <c r="J21" s="9">
         <v>0</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L21" s="9">
         <v>170</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="N21" s="9">
         <v>0</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P21" s="9">
         <v>0</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="R21" s="9">
         <v>9</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="T21" s="9">
         <v>35</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="V21" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W21" s="10" t="s">
-        <v>154</v>
+        <v>256</v>
       </c>
       <c r="X21" s="9">
         <v>37</v>
       </c>
       <c r="Y21" s="10" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="Z21" s="9">
         <v>39</v>
       </c>
       <c r="AA21" s="10" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="AB21" s="9">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AC21" s="10" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="AD21" s="9">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="AE21" s="10" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="AF21" s="9">
         <v>3</v>
       </c>
       <c r="AG21" s="10" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="AH21" s="9">
         <v>0</v>
       </c>
       <c r="AI21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ21" s="9">
         <v>119</v>
       </c>
       <c r="AK21" s="10" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="AL21" s="9">
         <v>384</v>
       </c>
       <c r="AM21" s="10" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="AN21" s="9">
         <v>0</v>
       </c>
       <c r="AO21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AP21" s="9">
         <v>0</v>
       </c>
       <c r="AQ21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR21" s="9">
         <v>0</v>
       </c>
       <c r="AS21" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C22" s="12">
-        <v>58216</v>
+        <v>60113</v>
       </c>
       <c r="D22" s="12">
         <v>7</v>
@@ -4049,7 +4040,7 @@
         <v>94</v>
       </c>
       <c r="F22" s="12">
-        <v>2441</v>
+        <v>2528</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>95</v>
@@ -4061,94 +4052,94 @@
         <v>96</v>
       </c>
       <c r="J22" s="12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K22" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="L22" s="12">
+        <v>12044</v>
+      </c>
+      <c r="M22" s="13" t="s">
         <v>97</v>
-      </c>
-      <c r="L22" s="12">
-        <v>11446</v>
-      </c>
-      <c r="M22" s="13" t="s">
-        <v>98</v>
       </c>
       <c r="N22" s="12">
         <v>3</v>
       </c>
       <c r="O22" s="13" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="P22" s="12">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="Q22" s="13" t="s">
         <v>99</v>
       </c>
       <c r="R22" s="12">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="S22" s="13" t="s">
         <v>100</v>
       </c>
       <c r="T22" s="12">
-        <v>1423</v>
+        <v>1443</v>
       </c>
       <c r="U22" s="13" t="s">
         <v>101</v>
       </c>
       <c r="V22" s="12">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="W22" s="13" t="s">
         <v>102</v>
       </c>
       <c r="X22" s="12">
-        <v>1670</v>
+        <v>1735</v>
       </c>
       <c r="Y22" s="13" t="s">
         <v>103</v>
       </c>
       <c r="Z22" s="12">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="AA22" s="13" t="s">
         <v>104</v>
       </c>
       <c r="AB22" s="12">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="AC22" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="AD22" s="12">
+        <v>26070</v>
+      </c>
+      <c r="AE22" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="AD22" s="12">
-        <v>25193</v>
-      </c>
-      <c r="AE22" s="13" t="s">
+      <c r="AF22" s="12">
+        <v>607</v>
+      </c>
+      <c r="AG22" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="AF22" s="12">
-        <v>603</v>
-      </c>
-      <c r="AG22" s="13" t="s">
+      <c r="AH22" s="12">
+        <v>12</v>
+      </c>
+      <c r="AI22" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="AH22" s="12">
-        <v>14</v>
-      </c>
-      <c r="AI22" s="13" t="s">
+      <c r="AJ22" s="12">
+        <v>9930</v>
+      </c>
+      <c r="AK22" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="AJ22" s="12">
-        <v>9655</v>
-      </c>
-      <c r="AK22" s="13" t="s">
+      <c r="AL22" s="12">
+        <v>4072</v>
+      </c>
+      <c r="AM22" s="13" t="s">
         <v>109</v>
-      </c>
-      <c r="AL22" s="12">
-        <v>4070</v>
-      </c>
-      <c r="AM22" s="13" t="s">
-        <v>110</v>
       </c>
       <c r="AN22" s="12">
         <v>4</v>
@@ -4160,13 +4151,13 @@
         <v>0</v>
       </c>
       <c r="AQ22" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AR22" s="12">
         <v>26</v>
       </c>
       <c r="AS22" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>